<commit_message>
Config: remove autopay from recourse paths, add recourse target score 495
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/actionability_table_en.xlsx
+++ b/reports/actionability_table_en.xlsx
@@ -1689,7 +1689,7 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>Varied</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>Can be changed immediately, creating an 'easy path'. But setting autopay does not lower real risk, so there is a gaming concern. Team to decide on inclusion in paths. Update: still open, classified ACTIONABLE for now. Step 3: 6-step discrete marginal, latent correlation -0.35, credit-link weight 0.5.</t>
+          <t>Can be changed immediately, creating an 'easy path'. But setting autopay does not lower real risk, so there is a gaming concern. Team to decide on inclusion in paths. Step 3: 6-step discrete marginal, latent correlation -0.35, credit-link weight 0.5. Decision (after the audit): removed from recourse paths (dice_vary: false) because setting up autopay does not lower real risk. Kept as a model feature. In the audit it was the easiest single path for 4,318 rejected applicants (about 2.5 months).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Config: reclassify autopay as NOT_RECOMMENDED
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/actionability_table_en.xlsx
+++ b/reports/actionability_table_en.xlsx
@@ -1633,73 +1633,73 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>autopay_ratio</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Share of recurring bills on autopay</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Simulated</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>ACTIONABLE</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Actionable</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>NOT_RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Not recommended</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Increase</t>
         </is>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="G19" s="8" t="n">
         <v>0.2</v>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>[0.0, 1.0]</t>
         </is>
       </c>
-      <c r="I19" s="4" t="n">
+      <c r="I19" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J19" s="4" t="n">
+      <c r="J19" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K19" s="8" t="inlineStr">
         <is>
           <t>-1 (higher value, lower PD)</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>Included in approval paths</t>
-        </is>
-      </c>
-      <c r="O19" s="4" t="inlineStr">
-        <is>
-          <t>Can be changed immediately, creating an 'easy path'. But setting autopay does not lower real risk, so there is a gaming concern. Team to decide on inclusion in paths. Step 3: 6-step discrete marginal, latent correlation -0.35, credit-link weight 0.5. Decision (after the audit): removed from recourse paths (dice_vary: false) because setting up autopay does not lower real risk. Kept as a model feature. In the audit it was the easiest single path for 4,318 rejected applicants (about 2.5 months).</t>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>Fixed in DiCE</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="inlineStr">
+        <is>
+          <t>Can be changed immediately, creating an 'easy path'. But setting autopay does not lower real risk, so there is a gaming concern. Team to decide on inclusion in paths. Step 3: 6-step discrete marginal, latent correlation -0.35, credit-link weight 0.5. Decision (after the audit): removed from recourse paths (dice_vary: false) because setting up autopay does not lower real risk. Kept as a model feature. In the audit it was the easiest single path for 4,318 rejected applicants (about 2.5 months). Then reclassified as NOT_RECOMMENDED. Monotone stays -1, so the final model is unchanged. Shown as 'reference (not changeable)' in SHAP rejection reasons.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Step 1: mission alternative variables, shared factor, renames
- Rename telecom/utility_ontime_rate to telecom/utility_payment_rate (mission names).
- Add spending_consistency, regular_payment_count, app_login_frequency to the copula.
- Mission variables calibrated to observed Pearson r -0.32; extras stay at latent 0.35.
- Shared factor for the 5 mission variables, largest pair kept at or below 0.60.
- Count variables use Binomial(n, 0.75) to avoid Poisson low-tail bunching.
- autopay_ratio: model_feature false (gameable); new model_feature field in the YAML and Excel.
- Retrained models and rebuilt MLflow under the new repo path.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/actionability_table_en.xlsx
+++ b/reports/actionability_table_en.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -499,8 +499,9 @@
     <col width="26" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="34" customWidth="1" min="14" max="14"/>
-    <col width="90" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="90" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -585,10 +586,15 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
+          <t>Model feature</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
           <t>Recourse handling</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -656,10 +662,15 @@
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
           <t>Included in approval paths</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>Can be lowered by paying down card and credit line balances. Time per step assumes a 0.05 decrease. Update (Step 1): the original plan was to clip values above 1 to 1; instead, values above 1 are kept (over-limit use is realistic) and only values above 10 are treated as errors (set missing, util_outlier flag). Bounds widened to [0, 10] to match. Step 2: default rate rises from about 1.4% to 23.4% across deciles.</t>
         </is>
@@ -733,10 +744,15 @@
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
           <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>Protected attribute. Immutable, so no monotonic constraint needed (a constraint would only cost AUC). Update: decided to use it as a model feature without a monotonic constraint. The one row with age = 0 was dropped in Step 1. Fairness note: age correlates with utilization (-0.28) and dependents (-0.23), and weakly with the alternative variables (0.05 to 0.09), so removing age alone would not remove age effects.</t>
         </is>
@@ -810,10 +826,15 @@
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
           <t>Fixed in DiCE</t>
         </is>
       </c>
-      <c r="O7" s="6" t="inlineStr">
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>Charter rule applies: late-payment history cannot decrease. It could drop over time due to the 2-year window, but is fixed in v1. Update (Step 1): codes 96/98 (269 rows, always in all three columns together) set to missing and flagged in pastdue_special_code (default rate 54.65%).</t>
         </is>
@@ -881,10 +902,15 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
           <t>Included with a high cost</t>
         </is>
       </c>
-      <c r="O8" s="7" t="inlineStr">
+      <c r="P8" s="7" t="inlineStr">
         <is>
           <t>Requires paying down debt or raising income. Rows with missing MonthlyIncome have abnormally large values. Update: Step 1 sets it to missing when income is missing or 0 (raw amounts, not ratios). Step 2 found a U shape, the weakest direction evidence, so it was first in the drop order. Step 5: the constraint cost only 0.0001 AUC, so +1 was kept.</t>
         </is>
@@ -954,10 +980,15 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
           <t>Included with a high cost</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr">
+      <c r="P9" s="7" t="inlineStr">
         <is>
           <t>Changeable but depends on external factors (employment). Step defined as a percentage (5%) to avoid currency issues. Update (Step 1): missing values (19.8%) kept as missing with the income_missing flag; 0 kept as a real value with the income_zero flag. Imputation (median) is fit on training folds only.</t>
         </is>
@@ -1031,10 +1062,15 @@
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
           <t>Fixed in DiCE</t>
         </is>
       </c>
-      <c r="O10" s="8" t="inlineStr">
+      <c r="P10" s="8" t="inlineStr">
         <is>
           <t>U-shaped relationship with default, so no direction constraint. Closing a card raises utilization; suggesting new accounts is inappropriate. Excluded from v1 paths. Update: Step 2 confirmed the U shape (highest default rate at 3 or fewer lines). Also used in the thin-filer rule (2 or fewer lines and 0 real estate loans).</t>
         </is>
@@ -1108,10 +1144,15 @@
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
           <t>Fixed in DiCE</t>
         </is>
       </c>
-      <c r="O11" s="6" t="inlineStr">
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>Cumulative history with no time window. Cannot decrease. Update: codes 96/98 handled as for the 30 to 59 day column. Strongest real predictor (Pearson r 0.315).</t>
         </is>
@@ -1185,10 +1226,15 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
           <t>Fixed in DiCE</t>
         </is>
       </c>
-      <c r="O12" s="8" t="inlineStr">
+      <c r="P12" s="8" t="inlineStr">
         <is>
           <t>Suggesting a mortgage as an approval path is unrealistic. Non-monotonic relationship. Update: Step 2 confirmed the U shape. Also used in the thin-filer rule.</t>
         </is>
@@ -1262,10 +1308,15 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
           <t>Fixed in DiCE</t>
         </is>
       </c>
-      <c r="O13" s="6" t="inlineStr">
+      <c r="P13" s="6" t="inlineStr">
         <is>
           <t>Same rule as 30 to 59 days past due.</t>
         </is>
@@ -1339,10 +1390,15 @@
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
           <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr">
+      <c r="P14" s="5" t="inlineStr">
         <is>
           <t>Advising someone to change family size is unethical, so treated as immutable. Update: 2.6% missing, imputed with the training-fold median.</t>
         </is>
@@ -1351,7 +1407,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>telecom_ontime_rate</t>
+          <t>telecom_payment_rate</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1410,19 +1466,24 @@
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
           <t>Included in approval paths</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr">
-        <is>
-          <t>Rises by 1/12 for each month paid on time. Suggested distribution: Beta. Target correlation -0.3 to -0.5. Update (Step 3): Beta(8, 1.5) marginal, copula latent correlation -0.35, observed Pearson -0.27. Linked to credit behavior (weight 1.0, b = 0.30).</t>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>Rises by 1/12 for each month paid on time. Suggested distribution: Beta. Target correlation -0.3 to -0.5. Update (Step 3): Beta(8, 1.5) marginal, copula latent correlation -0.35, observed Pearson -0.27. Linked to credit behavior (weight 1.0, b = 0.30). Update (mission compliance): renamed from telecom_ontime_rate to the mission name. Calibrated to observed Pearson r -0.32 and shares a common factor with the other mission variables.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>utility_ontime_rate</t>
+          <t>utility_payment_rate</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1481,12 +1542,17 @@
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
           <t>Included in approval paths</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
-        <is>
-          <t>Likely highly correlated with the phone bill rate; check the correlation between them too. Target correlation -0.3 to -0.5. Update (Step 3): same setup as the phone bill rate. Correlation between the two is 0.19 (cap 0.60), so no extra noise was needed.</t>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>Likely highly correlated with the phone bill rate; check the correlation between them too. Target correlation -0.3 to -0.5. Update (Step 3): same setup as the phone bill rate. Correlation between the two is 0.19 (cap 0.60), so no extra noise was needed. Update (mission compliance): renamed from utility_ontime_rate to the mission name. Calibrated to observed Pearson r -0.32 and shares a common factor with the other mission variables.</t>
         </is>
       </c>
     </row>
@@ -1552,10 +1618,15 @@
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
+        <is>
           <t>If included, reflect duration only; do not phrase as an action</t>
         </is>
       </c>
-      <c r="O17" s="9" t="inlineStr">
+      <c r="P17" s="9" t="inlineStr">
         <is>
           <t>Cannot be sped up by action; increases only with time. Suggested distribution: Gamma or lognormal. Update (Step 3): Gamma(2, 24) marginal, capped at (age - 18) x 12 months (applies to 0.69% of rows). Correlation with age 0.065. Credit-link weight 0.5.</t>
         </is>
@@ -1623,10 +1694,15 @@
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
           <t>If included, reflect duration only; do not phrase as an action</t>
         </is>
       </c>
-      <c r="O18" s="9" t="inlineStr">
+      <c r="P18" s="9" t="inlineStr">
         <is>
           <t>Requires enrollment (employment or regional). Increases only with time. A type of variable used in Korean alternative credit scoring. Update (Step 3): Binomial(24, 0.75) marginal, latent correlation -0.35, credit-link weight 0.5.</t>
         </is>
@@ -1694,255 +1770,257 @@
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="inlineStr">
+        <is>
           <t>Fixed in DiCE</t>
         </is>
       </c>
-      <c r="O19" s="8" t="inlineStr">
-        <is>
-          <t>Can be changed immediately, creating an 'easy path'. But setting autopay does not lower real risk, so there is a gaming concern. Team to decide on inclusion in paths. Step 3: 6-step discrete marginal, latent correlation -0.35, credit-link weight 0.5. Decision (after the audit): removed from recourse paths (dice_vary: false) because setting up autopay does not lower real risk. Kept as a model feature. In the audit it was the easiest single path for 4,318 rejected applicants (about 2.5 months). Then reclassified as NOT_RECOMMENDED. Monotone stays -1, so the final model is unchanged. Shown as 'reference (not changeable)' in SHAP rejection reasons.</t>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t>Can be changed immediately, creating an 'easy path'. But setting autopay does not lower real risk, so there is a gaming concern. Team to decide on inclusion in paths. Step 3: 6-step discrete marginal, latent correlation -0.35, credit-link weight 0.5. Decision (after the audit): removed from recourse paths (dice_vary: false) because setting up autopay does not lower real risk. Kept as a model feature. In the audit it was the easiest single path for 4,318 rejected applicants (about 2.5 months). Then reclassified as NOT_RECOMMENDED. Monotone stays -1, so the final model is unchanged. Shown as 'reference (not changeable)' in SHAP rejection reasons. Update (mission compliance): also excluded from the model features (model_feature: false) so a gameable variable does not drive decisions. It stays in the dataset.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>pastdue_special_code</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Past-due special code (96/98) flag</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Derived (Step 1)</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>IMMUTABLE</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Immutable</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K20" s="5" t="inlineStr">
-        <is>
-          <t>0 (none)</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>spending_consistency</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Spending consistency score (0 to 100)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Simulated</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>ACTIONABLE</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Increase</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>[0.0, 100.0]</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>-1 (higher value, lower PD)</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>Varied</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>Included in approval paths</t>
+        </is>
+      </c>
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>Mission alternative variable. Higher when monthly spending is steadier. Can be raised by changing spending habits, so actionable. Step size (5 points), difficulty (2) and months per step (1) are team assumptions that need mentor review. Simulated as Beta(5, 2) x 100, observed Pearson r -0.32, shares the common factor, credit-link weight 0.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>regular_payment_count</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Number of recurring payments (0 to 20)</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Simulated</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>NOT_RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Not recommended</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Increase</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>[0.0, 20.0]</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>-1 (higher value, lower PD)</t>
+        </is>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="N20" s="5" t="inlineStr">
-        <is>
-          <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>Added in Step 1. Marks the 269 rows where all three past-due columns hold 96/98 (special codes, not counts). Default rate 54.65%, so it carries strong signal. Derived from history, so immutable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>income_missing</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Monthly income missing flag</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Derived (Step 1)</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>IMMUTABLE</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Immutable</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>0 (none)</t>
-        </is>
-      </c>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O21" s="8" t="inlineStr">
+        <is>
+          <t>Fixed in DiCE</t>
+        </is>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Mission alternative variable. Adding recurring payments is easy to game and does not lower real risk (same reason as autopay), so not recommended and excluded from paths. Still a model feature. Simulated as Binomial(20, 0.75), 0 to 20, observed Pearson r -0.32, shares the common factor. Unlike the mission example, not linked to income.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>app_login_frequency</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>App login frequency (0 to 30)</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Simulated</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>NOT_RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Not recommended</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Increase</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>[0.0, 30.0]</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>-1 (higher value, lower PD)</t>
+        </is>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="N21" s="5" t="inlineStr">
-        <is>
-          <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
-        </is>
-      </c>
-      <c r="O21" s="5" t="inlineStr">
-        <is>
-          <t>Added in Step 1. Marks 29,731 rows (19.8%) with missing income. DebtRatio is also set to missing there because it holds raw amounts. Default rate 5.6%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>income_zero</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Monthly income equals zero flag</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Derived (Step 1)</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>IMMUTABLE</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Immutable</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K22" s="5" t="inlineStr">
-        <is>
-          <t>0 (none)</t>
-        </is>
-      </c>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M22" s="5" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="N22" s="5" t="inlineStr">
-        <is>
-          <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr">
-        <is>
-          <t>Added in Step 1. Marks 1,634 rows with income = 0 (kept as a real value). DebtRatio set to missing there. Default rate 4.0%.</t>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O22" s="8" t="inlineStr">
+        <is>
+          <t>Fixed in DiCE</t>
+        </is>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Mission alternative variable. Logging in more is pure gaming, so not recommended and excluded from paths. Still a model feature. The mission example links it to age; it is deliberately not linked to age, a protected attribute (the credit part uses only past-due counts and utilization). Simulated as Binomial(30, 0.75), 0 to 30 (days with a login), observed Pearson r -0.32, shares the common factor.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>util_outlier</t>
+          <t>pastdue_special_code</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Revolving utilization outlier (above 10) flag</t>
+          <t>Past-due special code (96/98) flag</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -2002,87 +2080,343 @@
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
           <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
         </is>
       </c>
-      <c r="O23" s="5" t="inlineStr">
-        <is>
-          <t>Added in Step 1. Marks 241 rows with utilization above 10 (treated as data errors, set to missing). Default rate 7.05%, close to average, so the simulator gives them a neutral credit score.</t>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>Added in Step 1. Marks the 269 rows where all three past-due columns hold 96/98 (special codes, not counts). Default rate 54.65%, so it carries strong signal. Derived from history, so immutable.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>income_missing</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Monthly income missing flag</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Derived (Step 1)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>IMMUTABLE</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Immutable</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>0 (none)</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>Added in Step 1. Marks 29,731 rows (19.8%) with missing income. DebtRatio is also set to missing there because it holds raw amounts. Default rate 5.6%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>income_zero</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Monthly income equals zero flag</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Derived (Step 1)</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>IMMUTABLE</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Immutable</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>0 (none)</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>Added in Step 1. Marks 1,634 rows with income = 0 (kept as a real value). DebtRatio set to missing there. Default rate 4.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>util_outlier</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Revolving utilization outlier (above 10) flag</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Derived (Step 1)</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>IMMUTABLE</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Immutable</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>0 (none)</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
+        </is>
+      </c>
+      <c r="P26" s="5" t="inlineStr">
+        <is>
+          <t>Added in Step 1. Marks 241 rows with utilization above 10 (treated as data errors, set to missing). Default rate 7.05%, close to average, so the simulator gives them a neutral credit score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
           <t>gender_female</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Gender (female = 1, simulated)</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Simulated</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>IMMUTABLE</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Immutable</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
         <is>
           <t>0 (none)</t>
         </is>
       </c>
-      <c r="L24" s="5" t="inlineStr">
+      <c r="L27" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M24" s="5" t="inlineStr">
+      <c r="M27" s="5" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="N24" s="5" t="inlineStr">
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="inlineStr">
         <is>
           <t>Fixed in DiCE; shown as 'reference (not changeable)' in rejection reasons</t>
         </is>
       </c>
-      <c r="O24" s="5" t="inlineStr">
+      <c r="P27" s="5" t="inlineStr">
         <is>
           <t>Added in Step 3. Simulated 50/50, independent of default (r = 0.0007). Used only for fairness analysis, never as a model feature. Protected attribute.</t>
         </is>

</xml_diff>